<commit_message>
Feature/memberManage: 헬스장 회원 관리 기능 추가
- GymMemberManage 페이지 신규 추가 (목록 조회·검색·삭제)
- /memberships/gyms/{gymId}/members GET·DELETE 엔드포인트 추가
- SecurityConfig에서 OWNER 역할도 /memberships/** 접근 허용
- docker-compose gemma4-ai를 선택적 profile로 분리

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Functional_Specification.xlsx
+++ b/Functional_Specification.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\finem\Desktop\gymbarofit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{397E504B-AE5E-42E0-9BC4-8221F8EDF9C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2909ADE1-15F8-4526-AA09-950B03DBF1B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1305" yWindow="1335" windowWidth="28770" windowHeight="15450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="129">
   <si>
     <t>기능 명세서</t>
   </si>
@@ -90,12 +90,6 @@
   </si>
   <si>
     <t>소셜 로그인 연동</t>
-  </si>
-  <si>
-    <t>미구현</t>
-  </si>
-  <si>
-    <t>추후 구현 예정</t>
   </si>
   <si>
     <t>역할 분리</t>
@@ -457,6 +451,14 @@
   </si>
   <si>
     <t>recharts 사용 (BarChart, PieChart) / visitByHour / lockerZoneUsage / equipmentUsage / monthlyEquipmentUsage</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>보류</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>구현</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -464,7 +466,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -518,8 +520,40 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -542,12 +576,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -598,8 +626,23 @@
         <bgColor rgb="FFE3F2FD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -646,11 +689,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -661,41 +728,50 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="4" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="4">
+    <cellStyle name="메모" xfId="2" builtinId="10"/>
+    <cellStyle name="보통" xfId="1" builtinId="28"/>
+    <cellStyle name="좋음" xfId="3" builtinId="26"/>
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1008,14 +1084,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
     </row>
     <row r="2" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -1038,7 +1114,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="16" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -1056,7 +1132,7 @@
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="8"/>
+      <c r="A4" s="9"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
         <v>12</v>
@@ -1070,7 +1146,7 @@
       <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8"/>
+      <c r="A5" s="9"/>
       <c r="B5" s="2" t="s">
         <v>14</v>
       </c>
@@ -1086,7 +1162,7 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8"/>
+      <c r="A6" s="9"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
         <v>17</v>
@@ -1100,7 +1176,7 @@
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
+      <c r="A7" s="9"/>
       <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
@@ -1110,119 +1186,117 @@
       <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="9"/>
+      <c r="B8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
-      <c r="B8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="E8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="9"/>
+      <c r="B9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
-      <c r="B9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="8"/>
+      <c r="A10" s="9"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="9"/>
+      <c r="B11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="8"/>
-      <c r="B11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="E11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>35</v>
-      </c>
     </row>
     <row r="12" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="9"/>
+      <c r="A12" s="10"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="2" t="s">
+    </row>
+    <row r="13" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
+      <c r="C13" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="8"/>
+      <c r="A14" s="9"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
@@ -1230,13 +1304,13 @@
       <c r="F14" s="2"/>
     </row>
     <row r="15" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="8"/>
+      <c r="A15" s="9"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
@@ -1244,13 +1318,13 @@
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="8"/>
+      <c r="A16" s="9"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
@@ -1258,13 +1332,13 @@
       <c r="F16" s="2"/>
     </row>
     <row r="17" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="8"/>
+      <c r="A17" s="9"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>11</v>
@@ -1272,75 +1346,75 @@
       <c r="F17" s="2"/>
     </row>
     <row r="18" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="8"/>
+      <c r="A18" s="9"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="2"/>
+    </row>
+    <row r="19" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="9"/>
+      <c r="B19" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="C19" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="8"/>
-      <c r="B19" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F19" s="2"/>
     </row>
     <row r="20" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="8"/>
+      <c r="A20" s="9"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>57</v>
-      </c>
     </row>
     <row r="21" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="8"/>
+      <c r="A21" s="9"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>60</v>
-      </c>
     </row>
     <row r="22" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="8"/>
+      <c r="A22" s="9"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>11</v>
@@ -1348,47 +1422,47 @@
       <c r="F22" s="2"/>
     </row>
     <row r="23" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="9"/>
+      <c r="A23" s="10"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="2"/>
+    </row>
+    <row r="24" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E23" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23" s="2"/>
-    </row>
-    <row r="24" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="14" t="s">
+      <c r="C24" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="E24" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>69</v>
-      </c>
     </row>
     <row r="25" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="8"/>
+      <c r="A25" s="9"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>11</v>
@@ -1396,45 +1470,45 @@
       <c r="F25" s="2"/>
     </row>
     <row r="26" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="9"/>
+      <c r="A26" s="10"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="2"/>
+    </row>
+    <row r="27" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="B27" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E26" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F26" s="2"/>
-    </row>
-    <row r="27" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="16" t="s">
+      <c r="C27" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="E27" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F27" s="2"/>
     </row>
     <row r="28" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="8"/>
+      <c r="A28" s="9"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>11</v>
@@ -1442,45 +1516,45 @@
       <c r="F28" s="2"/>
     </row>
     <row r="29" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="9"/>
+      <c r="A29" s="10"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="2"/>
+    </row>
+    <row r="30" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="B30" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E29" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F29" s="2"/>
-    </row>
-    <row r="30" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="10" t="s">
+      <c r="C30" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="D30" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="E30" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F30" s="2"/>
     </row>
     <row r="31" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="8"/>
+      <c r="A31" s="9"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>11</v>
@@ -1488,43 +1562,43 @@
       <c r="F31" s="2"/>
     </row>
     <row r="32" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="8"/>
+      <c r="A32" s="9"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="2"/>
+    </row>
+    <row r="33" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="9"/>
+      <c r="B33" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E32" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F32" s="2"/>
-    </row>
-    <row r="33" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="8"/>
-      <c r="B33" s="2" t="s">
+      <c r="D33" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="E33" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F33" s="2"/>
     </row>
     <row r="34" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="8"/>
+      <c r="A34" s="9"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>11</v>
@@ -1532,171 +1606,171 @@
       <c r="F34" s="2"/>
     </row>
     <row r="35" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="8"/>
+      <c r="A35" s="9"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="2"/>
+    </row>
+    <row r="36" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="9"/>
+      <c r="B36" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E35" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F35" s="2"/>
-    </row>
-    <row r="36" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="8"/>
-      <c r="B36" s="2" t="s">
+      <c r="D36" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>99</v>
-      </c>
       <c r="E36" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F36" s="2"/>
     </row>
     <row r="37" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="8"/>
+      <c r="A37" s="9"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" s="2"/>
+    </row>
+    <row r="38" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="9"/>
+      <c r="B38" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E37" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F37" s="2"/>
-    </row>
-    <row r="38" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="8"/>
-      <c r="B38" s="2" t="s">
+      <c r="D38" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="E38" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="F38" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>105</v>
-      </c>
     </row>
     <row r="39" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="9"/>
+      <c r="A39" s="10"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E39" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="F39" s="2"/>
+    </row>
+    <row r="40" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="B40" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E39" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F39" s="2"/>
-    </row>
-    <row r="40" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
+      <c r="C40" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="D40" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="E40" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D40" s="2" t="s">
+    </row>
+    <row r="41" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="E40" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F40" s="2" t="s">
+      <c r="B41" s="2" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="15" t="s">
+      <c r="C41" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="D41" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="E41" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" s="2"/>
+    </row>
+    <row r="42" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="9"/>
+      <c r="B42" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="C42" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E41" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F41" s="2"/>
-    </row>
-    <row r="42" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="8"/>
-      <c r="B42" s="2" t="s">
+      <c r="D42" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="E42" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="D42" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>120</v>
-      </c>
     </row>
     <row r="43" spans="1:6" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="9"/>
+      <c r="A43" s="10"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="D43" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="6" t="s">
+      <c r="C44" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="D44" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="E44" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feature/memberManage: 헬스장 회원 관리 기능 추가 (#19)
- GymMemberManage 페이지 신규 추가 (목록 조회·검색·삭제)
- /memberships/gyms/{gymId}/members GET·DELETE 엔드포인트 추가
- SecurityConfig에서 OWNER 역할도 /memberships/** 접근 허용
- docker-compose gemma4-ai를 선택적 profile로 분리

Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Functional_Specification.xlsx
+++ b/Functional_Specification.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\finem\Desktop\gymbarofit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{397E504B-AE5E-42E0-9BC4-8221F8EDF9C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2909ADE1-15F8-4526-AA09-950B03DBF1B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1305" yWindow="1335" windowWidth="28770" windowHeight="15450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="129">
   <si>
     <t>기능 명세서</t>
   </si>
@@ -90,12 +90,6 @@
   </si>
   <si>
     <t>소셜 로그인 연동</t>
-  </si>
-  <si>
-    <t>미구현</t>
-  </si>
-  <si>
-    <t>추후 구현 예정</t>
   </si>
   <si>
     <t>역할 분리</t>
@@ -457,6 +451,14 @@
   </si>
   <si>
     <t>recharts 사용 (BarChart, PieChart) / visitByHour / lockerZoneUsage / equipmentUsage / monthlyEquipmentUsage</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>보류</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>구현</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -464,7 +466,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -518,8 +520,40 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -542,12 +576,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -598,8 +626,23 @@
         <bgColor rgb="FFE3F2FD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -646,11 +689,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -661,41 +728,50 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="4" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="4">
+    <cellStyle name="메모" xfId="2" builtinId="10"/>
+    <cellStyle name="보통" xfId="1" builtinId="28"/>
+    <cellStyle name="좋음" xfId="3" builtinId="26"/>
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1008,14 +1084,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
     </row>
     <row r="2" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -1038,7 +1114,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="16" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -1056,7 +1132,7 @@
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="8"/>
+      <c r="A4" s="9"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
         <v>12</v>
@@ -1070,7 +1146,7 @@
       <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8"/>
+      <c r="A5" s="9"/>
       <c r="B5" s="2" t="s">
         <v>14</v>
       </c>
@@ -1086,7 +1162,7 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8"/>
+      <c r="A6" s="9"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
         <v>17</v>
@@ -1100,7 +1176,7 @@
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
+      <c r="A7" s="9"/>
       <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
@@ -1110,119 +1186,117 @@
       <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="9"/>
+      <c r="B8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
-      <c r="B8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="E8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="9"/>
+      <c r="B9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
-      <c r="B9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="8"/>
+      <c r="A10" s="9"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="9"/>
+      <c r="B11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="8"/>
-      <c r="B11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="E11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>35</v>
-      </c>
     </row>
     <row r="12" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="9"/>
+      <c r="A12" s="10"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="2" t="s">
+    </row>
+    <row r="13" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
+      <c r="C13" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="8"/>
+      <c r="A14" s="9"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
@@ -1230,13 +1304,13 @@
       <c r="F14" s="2"/>
     </row>
     <row r="15" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="8"/>
+      <c r="A15" s="9"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
@@ -1244,13 +1318,13 @@
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="8"/>
+      <c r="A16" s="9"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
@@ -1258,13 +1332,13 @@
       <c r="F16" s="2"/>
     </row>
     <row r="17" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="8"/>
+      <c r="A17" s="9"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>11</v>
@@ -1272,75 +1346,75 @@
       <c r="F17" s="2"/>
     </row>
     <row r="18" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="8"/>
+      <c r="A18" s="9"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="2"/>
+    </row>
+    <row r="19" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="9"/>
+      <c r="B19" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="C19" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="8"/>
-      <c r="B19" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F19" s="2"/>
     </row>
     <row r="20" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="8"/>
+      <c r="A20" s="9"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>57</v>
-      </c>
     </row>
     <row r="21" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="8"/>
+      <c r="A21" s="9"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>60</v>
-      </c>
     </row>
     <row r="22" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="8"/>
+      <c r="A22" s="9"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>11</v>
@@ -1348,47 +1422,47 @@
       <c r="F22" s="2"/>
     </row>
     <row r="23" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="9"/>
+      <c r="A23" s="10"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="2"/>
+    </row>
+    <row r="24" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E23" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23" s="2"/>
-    </row>
-    <row r="24" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="14" t="s">
+      <c r="C24" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="E24" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>69</v>
-      </c>
     </row>
     <row r="25" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="8"/>
+      <c r="A25" s="9"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>11</v>
@@ -1396,45 +1470,45 @@
       <c r="F25" s="2"/>
     </row>
     <row r="26" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="9"/>
+      <c r="A26" s="10"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="2"/>
+    </row>
+    <row r="27" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="B27" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E26" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F26" s="2"/>
-    </row>
-    <row r="27" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="16" t="s">
+      <c r="C27" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="E27" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F27" s="2"/>
     </row>
     <row r="28" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="8"/>
+      <c r="A28" s="9"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>11</v>
@@ -1442,45 +1516,45 @@
       <c r="F28" s="2"/>
     </row>
     <row r="29" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="9"/>
+      <c r="A29" s="10"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="2"/>
+    </row>
+    <row r="30" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="B30" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E29" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F29" s="2"/>
-    </row>
-    <row r="30" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="10" t="s">
+      <c r="C30" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="D30" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="E30" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F30" s="2"/>
     </row>
     <row r="31" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="8"/>
+      <c r="A31" s="9"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>11</v>
@@ -1488,43 +1562,43 @@
       <c r="F31" s="2"/>
     </row>
     <row r="32" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="8"/>
+      <c r="A32" s="9"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="2"/>
+    </row>
+    <row r="33" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="9"/>
+      <c r="B33" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E32" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F32" s="2"/>
-    </row>
-    <row r="33" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="8"/>
-      <c r="B33" s="2" t="s">
+      <c r="D33" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="E33" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F33" s="2"/>
     </row>
     <row r="34" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="8"/>
+      <c r="A34" s="9"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>11</v>
@@ -1532,171 +1606,171 @@
       <c r="F34" s="2"/>
     </row>
     <row r="35" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="8"/>
+      <c r="A35" s="9"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="2"/>
+    </row>
+    <row r="36" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="9"/>
+      <c r="B36" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E35" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F35" s="2"/>
-    </row>
-    <row r="36" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="8"/>
-      <c r="B36" s="2" t="s">
+      <c r="D36" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>99</v>
-      </c>
       <c r="E36" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F36" s="2"/>
     </row>
     <row r="37" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="8"/>
+      <c r="A37" s="9"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" s="2"/>
+    </row>
+    <row r="38" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="9"/>
+      <c r="B38" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E37" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F37" s="2"/>
-    </row>
-    <row r="38" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="8"/>
-      <c r="B38" s="2" t="s">
+      <c r="D38" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="E38" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="F38" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>105</v>
-      </c>
     </row>
     <row r="39" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="9"/>
+      <c r="A39" s="10"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E39" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="F39" s="2"/>
+    </row>
+    <row r="40" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="B40" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E39" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F39" s="2"/>
-    </row>
-    <row r="40" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
+      <c r="C40" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="D40" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="E40" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D40" s="2" t="s">
+    </row>
+    <row r="41" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="E40" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F40" s="2" t="s">
+      <c r="B41" s="2" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="15" t="s">
+      <c r="C41" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="D41" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="E41" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" s="2"/>
+    </row>
+    <row r="42" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="9"/>
+      <c r="B42" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="C42" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E41" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F41" s="2"/>
-    </row>
-    <row r="42" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="8"/>
-      <c r="B42" s="2" t="s">
+      <c r="D42" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="E42" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="D42" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>120</v>
-      </c>
     </row>
     <row r="43" spans="1:6" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="9"/>
+      <c r="A43" s="10"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="D43" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="6" t="s">
+      <c r="C44" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="D44" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="E44" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>